<commit_message>
wip(catalog): engine-style short names, owner listing, screenshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/catalog-import/catalog-fix-review.xlsx
+++ b/docs/catalog-import/catalog-fix-review.xlsx
@@ -30433,7 +30433,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1003 (5FT)</t>
+          <t>1003 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -30485,7 +30485,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1003 (3.5FT)</t>
+          <t>1003 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -30537,7 +30537,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1003 (3FT)</t>
+          <t>1003 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -30589,7 +30589,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1003 (200X200CM)</t>
+          <t>1003 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -30641,7 +30641,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1003 (220X220CM)</t>
+          <t>1003 BEDFRAME (220X220CM)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -30693,7 +30693,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1005 (6FT)</t>
+          <t>1005 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -30745,7 +30745,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1005 (5FT)</t>
+          <t>1005 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -30797,7 +30797,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1005 (3.5FT)</t>
+          <t>1005 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -30849,7 +30849,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1005 (3FT)</t>
+          <t>1005 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -30901,7 +30901,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1005 (200X200CM)</t>
+          <t>1005 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -30953,7 +30953,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1007 (152X200CM)</t>
+          <t>1007 BEDFRAME (152X200CM)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -31005,7 +31005,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1007 (153X200CM)</t>
+          <t>1007 BEDFRAME (153X200CM)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -31057,7 +31057,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1007 (183X200CM)</t>
+          <t>1007 BEDFRAME (183X200CM)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -31109,7 +31109,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1008 (6FT)</t>
+          <t>1008 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -31161,7 +31161,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1008 (5FT)</t>
+          <t>1008 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1008 (3.5FT)</t>
+          <t>1008 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -31265,7 +31265,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1008 (3FT)</t>
+          <t>1008 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -31317,7 +31317,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1009 (6FT)</t>
+          <t>1009 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -31369,7 +31369,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1009 (5FT)</t>
+          <t>1009 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -31421,7 +31421,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1009 (3.5FT)</t>
+          <t>1009 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1009 (3FT)</t>
+          <t>1009 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -31525,7 +31525,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1013 (6FT)</t>
+          <t>1013 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -31577,7 +31577,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1013 (5FT)</t>
+          <t>1013 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -31629,7 +31629,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1013 (3.5FT)</t>
+          <t>1013 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -31681,7 +31681,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1013 (3FT)</t>
+          <t>1013 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -31733,7 +31733,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1013 (200X200CM)</t>
+          <t>1013 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -31785,7 +31785,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1019 (6FT)</t>
+          <t>1019 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -31837,7 +31837,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1019 (5FT)</t>
+          <t>1019 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -31889,7 +31889,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1019 (3.5FT)</t>
+          <t>1019 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -31941,7 +31941,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1019 (3FT)</t>
+          <t>1019 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -31993,7 +31993,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1023 (6FT)</t>
+          <t>1023 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -32045,7 +32045,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1023 (5FT)</t>
+          <t>1023 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -32097,7 +32097,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1023 (3.5FT)</t>
+          <t>1023 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -32149,7 +32149,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1023 (3FT)</t>
+          <t>1023 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -32201,7 +32201,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1030 (6FT)</t>
+          <t>1030 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -32253,7 +32253,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1030 (5FT)</t>
+          <t>1030 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -32305,7 +32305,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1030 (3.5FT)</t>
+          <t>1030 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -32357,7 +32357,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1030 (3FT)</t>
+          <t>1030 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -32409,7 +32409,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1030 (153X200CM)</t>
+          <t>1030 BEDFRAME (153X200CM)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -32461,7 +32461,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1041 (6FT)</t>
+          <t>1041 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -32513,7 +32513,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1041 (5FT)</t>
+          <t>1041 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1041 (3.5FT)</t>
+          <t>1041 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -32617,7 +32617,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1041 (3FT)</t>
+          <t>1041 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -32669,7 +32669,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1041 (107X200CM)</t>
+          <t>1041 BEDFRAME (107X200CM)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -32721,7 +32721,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1051 (6FT)</t>
+          <t>1051 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -32773,7 +32773,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1052 (6FT)</t>
+          <t>1052 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -32825,7 +32825,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1052 (5FT)</t>
+          <t>1052 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -32877,7 +32877,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 1052 (3.5FT)</t>
+          <t>1052 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -32929,7 +32929,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2003 (6FT)</t>
+          <t>2003 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -32981,7 +32981,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2003 (5FT)</t>
+          <t>2003 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -33033,7 +33033,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2003 (3.5FT)</t>
+          <t>2003 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -33085,7 +33085,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2003 (3FT)</t>
+          <t>2003 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -33137,7 +33137,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2003 (183X200CM)</t>
+          <t>2003 BEDFRAME (183X200CM)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -33189,7 +33189,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2006 (5FT)</t>
+          <t>2006 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -33241,7 +33241,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2006 (3.5FT)</t>
+          <t>2006 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -33293,7 +33293,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2006 (3FT)</t>
+          <t>2006 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -33345,7 +33345,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2006 (200X200CM)</t>
+          <t>2006 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -33397,7 +33397,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2006 (190X200CM)</t>
+          <t>2006 BEDFRAME (190X200CM)</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -33449,7 +33449,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2008 (200X200CM)</t>
+          <t>2008 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -33501,7 +33501,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2008 (152X200CM)</t>
+          <t>2008 BEDFRAME (152X200CM)</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2008 (183X200CM)</t>
+          <t>2008 BEDFRAME (183X200CM)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -33605,7 +33605,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2009 (200X200CM)</t>
+          <t>2009 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -33657,7 +33657,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2009 (152X200CM)</t>
+          <t>2009 BEDFRAME (152X200CM)</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -33709,7 +33709,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2009 (210X210CM)</t>
+          <t>2009 BEDFRAME (210X210CM)</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -33761,7 +33761,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2010 (6FT)</t>
+          <t>2010 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -33813,7 +33813,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2010 (5FT)</t>
+          <t>2010 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -33865,7 +33865,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2010 (3.5FT)</t>
+          <t>2010 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -33917,7 +33917,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2010 (3FT)</t>
+          <t>2010 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -33969,7 +33969,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2011 (6FT)</t>
+          <t>2011 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -34021,7 +34021,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2011 (5FT)</t>
+          <t>2011 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -34073,7 +34073,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2011 (3.5FT)</t>
+          <t>2011 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -34125,7 +34125,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2011 (3FT)</t>
+          <t>2011 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -34177,7 +34177,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2011 (200X200CM)</t>
+          <t>2011 BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -34229,7 +34229,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2023 (6FT)</t>
+          <t>2023 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -34281,7 +34281,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2023 (3FT)</t>
+          <t>2023 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -34333,7 +34333,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2027 (6FT)</t>
+          <t>2027 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -34385,7 +34385,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2027 (5FT)</t>
+          <t>2027 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2027 (3.5FT)</t>
+          <t>2027 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -34489,7 +34489,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2027 (3FT)</t>
+          <t>2027 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -34541,7 +34541,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2033 (6FT)</t>
+          <t>2033 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -34593,7 +34593,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2033 (5FT)</t>
+          <t>2033 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -34645,7 +34645,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2033 (3.5FT)</t>
+          <t>2033 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -34697,7 +34697,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2033 (3FT)</t>
+          <t>2033 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -34749,7 +34749,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2038 (6FT)</t>
+          <t>2038 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -34801,7 +34801,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2038 (5FT)</t>
+          <t>2038 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -34853,7 +34853,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2038 (3.5FT)</t>
+          <t>2038 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -34905,7 +34905,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2038 (3FT)</t>
+          <t>2038 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -34957,7 +34957,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2041 (6FT)</t>
+          <t>2041 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -35009,7 +35009,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2041 (5FT)</t>
+          <t>2041 BEDFRAME (5FT)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -35061,7 +35061,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2041 (3.5FT)</t>
+          <t>2041 BEDFRAME (3.5FT)</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -35113,7 +35113,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2041 (3FT)</t>
+          <t>2041 BEDFRAME (3FT)</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -35165,7 +35165,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME 2049 (6FT)</t>
+          <t>2049 BEDFRAME (6FT)</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -35217,7 +35217,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME DIVAN (200X200CM)</t>
+          <t>DIVAN BEDFRAME (200X200CM)</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -35269,7 +35269,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME DIVAN (153X210CM)</t>
+          <t>DIVAN BEDFRAME (153X210CM)</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -35321,7 +35321,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA BEDFRAME DIVAN (170X200CM)</t>
+          <t>DIVAN BEDFRAME (170X200CM)</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -35439,7 +35439,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5530 1A(LHF)</t>
+          <t>SOFA 5530 1A(LHF)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -35481,7 +35481,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5530 1A(RHF)</t>
+          <t>SOFA 5530 1A(RHF)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -35523,7 +35523,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5530 1NA</t>
+          <t>SOFA 5530 1NA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -35565,7 +35565,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5530 1S</t>
+          <t>SOFA 5530 1S</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -35607,7 +35607,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5530 2A(LHF)</t>
+          <t>SOFA 5530 2A(LHF)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -35649,7 +35649,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5531 XAMMAR 1A(LHF)</t>
+          <t>SOFA 5531 1A(LHF)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5531 XAMMAR 1A(RHF)</t>
+          <t>SOFA 5531 1A(RHF)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -35733,7 +35733,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5531 XAMMAR 1NA</t>
+          <t>SOFA 5531 1NA</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -35775,7 +35775,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5531 XAMMAR 1S</t>
+          <t>SOFA 5531 1S</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -35817,7 +35817,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5531 XAMMAR 2A(LHF)</t>
+          <t>SOFA 5531 2A(LHF)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -35859,7 +35859,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5535 TRRBU 1A(LHF)</t>
+          <t>SOFA 5535 1A(LHF)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -35901,7 +35901,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5535 TRRBU 1A(RHF)</t>
+          <t>SOFA 5535 1A(RHF)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -35943,7 +35943,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5535 TRRBU 1NA</t>
+          <t>SOFA 5535 1NA</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5535 TRRBU 1S</t>
+          <t>SOFA 5535 1S</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -36027,7 +36027,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5535 TRRBU 2A(LHF)</t>
+          <t>SOFA 5535 2A(LHF)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -36069,7 +36069,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5536 1A(LHF)</t>
+          <t>SOFA 5536 1A(LHF)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -36111,7 +36111,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5536 1A(RHF)</t>
+          <t>SOFA 5536 1A(RHF)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -36153,7 +36153,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5536 1NA</t>
+          <t>SOFA 5536 1NA</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -36195,7 +36195,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5536 1S</t>
+          <t>SOFA 5536 1S</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -36237,7 +36237,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5536 2A(LHF)</t>
+          <t>SOFA 5536 2A(LHF)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -36279,7 +36279,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5537 1A(LHF)</t>
+          <t>SOFA 5537 1A(LHF)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -36321,7 +36321,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5537 1A(RHF)</t>
+          <t>SOFA 5537 1A(RHF)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -36363,7 +36363,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5537 1NA</t>
+          <t>SOFA 5537 1NA</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -36405,7 +36405,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5537 1S</t>
+          <t>SOFA 5537 1S</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -36447,7 +36447,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5537 2A(LHF)</t>
+          <t>SOFA 5537 2A(LHF)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5539 BOOQIT 1A(LHF)</t>
+          <t>SOFA 5539 1A(LHF)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -36531,7 +36531,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5539 BOOQIT 1A(RHF)</t>
+          <t>SOFA 5539 1A(RHF)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -36573,7 +36573,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5539 BOOQIT 1B(LHF)</t>
+          <t>SOFA 5539 1B(LHF)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -36615,7 +36615,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5539 BOOQIT 1B(RHF)</t>
+          <t>SOFA 5539 1B(RHF)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -36657,7 +36657,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5539 BOOQIT 1NA</t>
+          <t>SOFA 5539 1NA</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -36699,7 +36699,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5540 1A(LHF)</t>
+          <t>SOFA 5540 1A(LHF)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -36741,7 +36741,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5540 1A(RHF)</t>
+          <t>SOFA 5540 1A(RHF)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5540 1NA</t>
+          <t>SOFA 5540 1NA</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -36825,7 +36825,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5540 1S</t>
+          <t>SOFA 5540 1S</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -36867,7 +36867,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5540 2A(LHF)</t>
+          <t>SOFA 5540 2A(LHF)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -36909,7 +36909,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5543 1B(LHF)</t>
+          <t>SOFA 5543 1B(LHF)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -36951,7 +36951,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5543 1B(RHF)</t>
+          <t>SOFA 5543 1B(RHF)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -36993,7 +36993,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5543 1NA</t>
+          <t>SOFA 5543 1NA</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -37035,7 +37035,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5543 1S</t>
+          <t>SOFA 5543 1S</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -37077,7 +37077,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5545 1A(LHF)</t>
+          <t>SOFA 5545 1A(LHF)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -37119,7 +37119,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5545 1A(RHF)</t>
+          <t>SOFA 5545 1A(RHF)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -37161,7 +37161,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5545 1B(LHF)</t>
+          <t>SOFA 5545 1B(LHF)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -37203,7 +37203,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5545 1B(RHF)</t>
+          <t>SOFA 5545 1B(RHF)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -37245,7 +37245,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5545 1NA</t>
+          <t>SOFA 5545 1NA</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5546 1A(LHF)</t>
+          <t>SOFA 5546 1A(LHF)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -37329,7 +37329,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5546 1A(RHF)</t>
+          <t>SOFA 5546 1A(RHF)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -37371,7 +37371,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5546 1B(LHF)</t>
+          <t>SOFA 5546 1B(LHF)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -37413,7 +37413,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5546 1B(RHF)</t>
+          <t>SOFA 5546 1B(RHF)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -37455,7 +37455,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5546 1NA</t>
+          <t>SOFA 5546 1NA</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5547 1A(LHF)</t>
+          <t>SOFA 5547 1A(LHF)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -37539,7 +37539,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5547 1A(RHF)</t>
+          <t>SOFA 5547 1A(RHF)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -37581,7 +37581,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5547 1B(LHF)</t>
+          <t>SOFA 5547 1B(LHF)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -37623,7 +37623,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5547 1B(RHF)</t>
+          <t>SOFA 5547 1B(RHF)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -37665,7 +37665,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5547 1NA</t>
+          <t>SOFA 5547 1NA</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -37707,7 +37707,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5548 1A(LHF)</t>
+          <t>SOFA 5548 1A(LHF)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -37749,7 +37749,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5548 1A(RHF)</t>
+          <t>SOFA 5548 1A(RHF)</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -37791,7 +37791,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5548 1B(LHF)</t>
+          <t>SOFA 5548 1B(LHF)</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -37833,7 +37833,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5548 1B(RHF)</t>
+          <t>SOFA 5548 1B(RHF)</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -37875,7 +37875,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5548 1NA</t>
+          <t>SOFA 5548 1NA</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -37917,7 +37917,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5549 1A(LHF)</t>
+          <t>SOFA 5549 1A(LHF)</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -37959,7 +37959,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5549 1A(RHF)</t>
+          <t>SOFA 5549 1A(RHF)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -38001,7 +38001,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5549 1B(LHF)</t>
+          <t>SOFA 5549 1B(LHF)</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -38043,7 +38043,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5549 1B(RHF)</t>
+          <t>SOFA 5549 1B(RHF)</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 5549 1NA</t>
+          <t>SOFA 5549 1NA</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -38127,7 +38127,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>HOOKKA SOFA 6112 2S</t>
+          <t>SOFA 6112 2S</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">

</xml_diff>